<commit_message>
kccn-sct-vn v1.17.2: hoan thien TMDT phu luc CCN - Bao Minh 500 ty (BC dau tu 14/10/2025, CSH 15% + BIDV 425 ty); nhom da thanh lap tong hop 1.360,01 ty (2/7 cum); quy tac khong tam tinh theo suat von
</commit_message>
<xml_diff>
--- a/kccn-sct-vn/skills/kccn-sct-vn/vi-du-thuc-te/2026.08.07. Danh mục thu hút đầu tư các CCN đến năm 2030 (theo QĐ số 1382).xlsx
+++ b/kccn-sct-vn/skills/kccn-sct-vn/vi-du-thuc-te/2026.08.07. Danh mục thu hút đầu tư các CCN đến năm 2030 (theo QĐ số 1382).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="179">
   <si>
     <t xml:space="preserve">DANH MỤC CÁC CỤM CÔNG NGHIỆP ĐÃ THÀNH LẬP VÀ THU HÚT ĐẦU TƯ HẠ TẦNG</t>
   </si>
@@ -86,6 +86,9 @@
     <t xml:space="preserve">Đã có Quyết định thành lập; giải phóng mặt bằng lũy kế 18/75 ha; vướng chồng lấn ranh giới với Công ty cổ phần Chè Văn Hưng. Cập nhật 06/8/2026: Sở Nông nghiệp và Môi trường đã thành lập Hội đồng thẩm định cấp Giấy phép môi trường Dự án đầu tư xây dựng kết cấu hạ tầng kỹ thuật cụm (QĐ 678/QĐ-SNNMT ngày 06/8/2026).</t>
   </si>
   <si>
+    <t xml:space="preserve">TMĐT: bổ sung theo QĐ chấp thuận CTĐT (hồ sơ gốc)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Phú Thịnh 2</t>
   </si>
   <si>
@@ -263,6 +266,9 @@
     <t xml:space="preserve">Thành lập tại QĐ 581/QĐ-UBND ngày 05/3/2026; chấp thuận chủ trương đầu tư đồng thời chấp thuận nhà đầu tư tại QĐ 1397/QĐ-UBND ngày 25/4/2026. Đang lập, trình duyệt Quy hoạch chi tiết 1/500; giải phóng mặt bằng 10/60 ha; phải chuyển đổi 12,87 ha đất rừng sản xuất.</t>
   </si>
   <si>
+    <t xml:space="preserve">TMĐT 500 tỷ theo Báo cáo đầu tư 14/10/2025 (vốn CSH 75 tỷ = 15%, BIDV cam kết tín dụng 425 tỷ) - đối chiếu bản gốc QĐ 1397/QĐ-UBND</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yên Hợp</t>
   </si>
   <si>
@@ -551,7 +557,7 @@
     <t xml:space="preserve">TỔNG CỘNG (I + II)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ghi chú: Danh mục và diện tích theo Phương án phát triển cụm công nghiệp kèm theo Quyết định số 525/QĐ-UBND ngày 25/02/2026 và Quyết định số 1382/QĐ-UBND ngày 23/4/2026 của UBND tỉnh Lào Cai. Trình tự thành lập, quản lý cụm công nghiệp thực hiện theo Nghị định số 32/2024/NĐ-CP, được sửa đổi, bổ sung tại Nghị định số 303/2026/NĐ-CP ngày 01/8/2026 của Chính phủ và Quyết định số 16/2026/QĐ-UBND của UBND tỉnh. Các nội dung ghi "(đề nghị xác nhận)", "(chưa xác định)" và các trường hợp diện tích còn hai số liệu khác nhau cần đối chiếu hồ sơ gốc trước khi đưa vào văn bản chính thức. Tổng mức đầu tư: 37 cụm giai đoạn 2026-2030 ghi theo Phụ lục 01 Quyết định 1382/QĐ-UBND ngày 23/4/2026 và Báo cáo Sở Công Thương ngày 18/6/2026 (suất vốn 7.611 triệu đồng/ha theo QĐ 425/QĐ-BXD); CCN Thống Nhất 1 ghi 860,008 tỷ đồng theo QĐ 298/QĐ-UBND ngày 20/02/2025 và QĐ 630/QĐ-UBND ngày 06/3/2025. Các cụm đã thành lập còn lại (Minh Quân, Phú Thịnh 1, 2, 3, Y Can, Bảo Minh) chưa có số liệu tổng mức đầu tư trong hồ sơ hiện có - đề nghị bổ sung Quyết định chấp thuận chủ trương đầu tư của từng cụm. Tiến độ cập nhật đến ngày 07/8/2026 theo sổ văn bản đến, văn bản đi của Sở.</t>
+    <t xml:space="preserve">Ghi chú: Danh mục và diện tích theo Phương án phát triển cụm công nghiệp kèm theo Quyết định số 525/QĐ-UBND ngày 25/02/2026 và Quyết định số 1382/QĐ-UBND ngày 23/4/2026 của UBND tỉnh Lào Cai. Trình tự thành lập, quản lý cụm công nghiệp thực hiện theo Nghị định số 32/2024/NĐ-CP, được sửa đổi, bổ sung tại Nghị định số 303/2026/NĐ-CP ngày 01/8/2026 của Chính phủ và Quyết định số 16/2026/QĐ-UBND của UBND tỉnh. Các nội dung ghi "(đề nghị xác nhận)", "(chưa xác định)" và các trường hợp diện tích còn hai số liệu khác nhau cần đối chiếu hồ sơ gốc trước khi đưa vào văn bản chính thức. Tổng mức đầu tư: 37 cụm giai đoạn 2026-2030 ghi theo Phụ lục 01 Quyết định 1382/QĐ-UBND ngày 23/4/2026 và Báo cáo Sở Công Thương ngày 18/6/2026 (suất vốn 7.611 triệu đồng/ha theo QĐ 425/QĐ-BXD); CCN Thống Nhất 1 ghi 860,008 tỷ đồng theo QĐ 298/QĐ-UBND ngày 20/02/2025 và QĐ 630/QĐ-UBND ngày 06/3/2025; CCN Bảo Minh ghi 500 tỷ đồng theo Báo cáo đầu tư ngày 14/10/2025 của Công ty CP Đầu tư Trung Chính Bảo Minh (đối chiếu bản gốc QĐ 1397/QĐ-UBND ngày 25/4/2026). Các cụm đã thành lập còn lại (Minh Quân, Phú Thịnh 1, 2, 3, Y Can) chưa có số liệu tổng mức đầu tư trong hồ sơ hiện có - đề nghị bổ sung Quyết định chấp thuận chủ trương đầu tư của từng cụm; KHÔNG tự tạm tính theo suất vốn để tránh lẫn với số liệu pháp lý. Tiến độ cập nhật đến ngày 07/8/2026 theo sổ văn bản đến, văn bản đi của Sở.</t>
   </si>
 </sst>
 </file>
@@ -958,8 +964,8 @@
     </row>
     <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="str">
-        <f aca="false">"Tổng số danh mục: 56 cụm công nghiệp (19 đã thành lập + 37 thành lập giai đoạn 2026-2030); tổng diện tích quy hoạch đến năm 2030: "&amp;TEXT(D71,"#,##0.00")&amp;" ha; tổng mức đầu tư dự kiến 37 cụm giai đoạn 2026-2030: "&amp;TEXT(E33,"#,##0.00")&amp;" tỷ đồng"</f>
-        <v>Tổng số danh mục: 56 cụm công nghiệp (19 đã thành lập + 37 thành lập giai đoạn 2026-2030); tổng diện tích quy hoạch đến năm 2030: 3,052.81 ha; tổng mức đầu tư dự kiến 37 cụm giai đoạn 2026-2030: 24,354.00 tỷ đồng</v>
+        <f aca="false">"Tổng số danh mục: 56 cụm công nghiệp (19 đã thành lập + 37 thành lập giai đoạn 2026-2030); tổng diện tích quy hoạch đến năm 2030: "&amp;TEXT(D71,"#,##0.00")&amp;" ha; tổng mức đầu tư dự kiến 37 cụm giai đoạn 2026-2030: "&amp;TEXT(E33,"#,##0.00")&amp;" tỷ đồng; nhóm cụm đã thành lập tổng hợp được "&amp;TEXT(E13,"#,##0.00")&amp;" tỷ đồng (02/07 cụm có chủ đầu tư đã có số liệu)"</f>
+        <v>Tổng số danh mục: 56 cụm công nghiệp (19 đã thành lập + 37 thành lập giai đoạn 2026-2030); tổng diện tích quy hoạch đến năm 2030: 3,052.81 ha; tổng mức đầu tư dự kiến 37 cụm giai đoạn 2026-2030: 24,354.00 tỷ đồng; nhóm cụm đã thành lập tổng hợp được 1,360.01 tỷ đồng (02/07 cụm có chủ đầu tư đã có số liệu)</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1067,7 +1073,7 @@
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">SUM(E14:E32)</f>
-        <v>860.008</v>
+        <v>1360.008</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
@@ -1093,14 +1099,16 @@
       <c r="G14" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="11"/>
-    </row>
-    <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H14" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="n">
         <v>2</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>18</v>
@@ -1110,19 +1118,21 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="11"/>
-    </row>
-    <row r="16" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>24</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="n">
         <v>3</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>18</v>
@@ -1132,32 +1142,34 @@
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H16" s="11"/>
+        <v>27</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="n">
         <v>4</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D17" s="10" t="n">
         <v>58.76</v>
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H17" s="11"/>
     </row>
@@ -1166,23 +1178,23 @@
         <v>5</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D18" s="10" t="n">
         <v>39.97</v>
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="72.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1190,20 +1202,20 @@
         <v>6</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D19" s="10" t="n">
         <v>20</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H19" s="11"/>
     </row>
@@ -1212,64 +1224,68 @@
         <v>7</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D20" s="10" t="n">
         <v>75</v>
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="H20" s="11"/>
-    </row>
-    <row r="21" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>42</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="n">
         <v>8</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D21" s="10" t="n">
         <v>75</v>
       </c>
       <c r="E21" s="10"/>
       <c r="F21" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="H21" s="11"/>
+        <v>46</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="n">
         <v>9</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D22" s="10" t="n">
         <v>55</v>
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H22" s="11"/>
     </row>
@@ -1278,20 +1294,20 @@
         <v>10</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D23" s="10" t="n">
         <v>31.01</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H23" s="11"/>
     </row>
@@ -1300,10 +1316,10 @@
         <v>11</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D24" s="10" t="n">
         <v>75</v>
@@ -1312,13 +1328,13 @@
         <v>860.008</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1326,23 +1342,23 @@
         <v>12</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D25" s="10" t="n">
         <v>17.17</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1350,23 +1366,23 @@
         <v>13</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D26" s="10" t="n">
         <v>19.5</v>
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1374,23 +1390,23 @@
         <v>14</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D27" s="10" t="n">
         <v>75</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="72.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1398,23 +1414,23 @@
         <v>15</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D28" s="10" t="n">
         <v>50</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1422,23 +1438,23 @@
         <v>16</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D29" s="10" t="n">
         <v>75</v>
       </c>
       <c r="E29" s="10"/>
       <c r="F29" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1446,77 +1462,81 @@
         <v>17</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D30" s="10" t="n">
         <v>60</v>
       </c>
       <c r="E30" s="10"/>
       <c r="F30" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="86.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="129.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="n">
         <v>18</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D31" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="E31" s="10"/>
+      <c r="E31" s="10" t="n">
+        <v>500</v>
+      </c>
       <c r="F31" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H31" s="11"/>
+        <v>80</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="72.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="n">
         <v>19</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D32" s="10" t="n">
         <v>12</v>
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="29.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7" t="n">
@@ -1536,10 +1556,10 @@
         <v>1</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D34" s="10" t="n">
         <v>75</v>
@@ -1548,10 +1568,10 @@
         <v>900</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H34" s="11"/>
     </row>
@@ -1560,10 +1580,10 @@
         <v>2</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D35" s="10" t="n">
         <v>50</v>
@@ -1572,10 +1592,10 @@
         <v>600</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H35" s="11"/>
     </row>
@@ -1584,10 +1604,10 @@
         <v>3</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>55</v>
@@ -1596,10 +1616,10 @@
         <v>660</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H36" s="11"/>
     </row>
@@ -1608,10 +1628,10 @@
         <v>4</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D37" s="10" t="n">
         <v>75</v>
@@ -1620,10 +1640,10 @@
         <v>900</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H37" s="11"/>
     </row>
@@ -1632,10 +1652,10 @@
         <v>5</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D38" s="10" t="n">
         <v>75</v>
@@ -1644,13 +1664,13 @@
         <v>900</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,7 +1678,7 @@
         <v>6</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>18</v>
@@ -1670,10 +1690,10 @@
         <v>900</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H39" s="11"/>
     </row>
@@ -1682,10 +1702,10 @@
         <v>7</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D40" s="10" t="n">
         <v>75</v>
@@ -1694,10 +1714,10 @@
         <v>900</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H40" s="11"/>
     </row>
@@ -1706,10 +1726,10 @@
         <v>8</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D41" s="10" t="n">
         <v>75</v>
@@ -1718,10 +1738,10 @@
         <v>900</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H41" s="11"/>
     </row>
@@ -1730,10 +1750,10 @@
         <v>9</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D42" s="10" t="n">
         <v>50</v>
@@ -1742,13 +1762,13 @@
         <v>600</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1756,10 +1776,10 @@
         <v>10</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D43" s="10" t="n">
         <v>63</v>
@@ -1768,13 +1788,13 @@
         <v>756</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1782,10 +1802,10 @@
         <v>11</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>37.4</v>
@@ -1794,10 +1814,10 @@
         <v>450</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H44" s="11"/>
     </row>
@@ -1806,10 +1826,10 @@
         <v>12</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D45" s="10" t="n">
         <v>75</v>
@@ -1818,10 +1838,10 @@
         <v>900</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H45" s="11"/>
     </row>
@@ -1830,10 +1850,10 @@
         <v>13</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D46" s="10" t="n">
         <v>20</v>
@@ -1842,10 +1862,10 @@
         <v>240</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G46" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H46" s="11"/>
     </row>
@@ -1854,10 +1874,10 @@
         <v>14</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D47" s="10" t="n">
         <v>40</v>
@@ -1866,13 +1886,13 @@
         <v>480</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1880,10 +1900,10 @@
         <v>15</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D48" s="10" t="n">
         <v>40</v>
@@ -1892,13 +1912,13 @@
         <v>480</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1906,10 +1926,10 @@
         <v>16</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D49" s="10" t="n">
         <v>35</v>
@@ -1918,10 +1938,10 @@
         <v>420</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H49" s="11"/>
     </row>
@@ -1930,10 +1950,10 @@
         <v>17</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D50" s="10" t="n">
         <v>75</v>
@@ -1942,10 +1962,10 @@
         <v>900</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G50" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H50" s="11"/>
     </row>
@@ -1954,10 +1974,10 @@
         <v>18</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D51" s="10" t="n">
         <v>75</v>
@@ -1966,10 +1986,10 @@
         <v>900</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H51" s="11"/>
     </row>
@@ -1978,10 +1998,10 @@
         <v>19</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D52" s="10" t="n">
         <v>57</v>
@@ -1990,10 +2010,10 @@
         <v>684</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G52" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H52" s="11"/>
     </row>
@@ -2002,10 +2022,10 @@
         <v>20</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D53" s="10" t="n">
         <v>30</v>
@@ -2014,13 +2034,13 @@
         <v>360</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2028,10 +2048,10 @@
         <v>21</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D54" s="10" t="n">
         <v>40</v>
@@ -2040,13 +2060,13 @@
         <v>480</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G54" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2054,10 +2074,10 @@
         <v>22</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D55" s="10" t="n">
         <v>20</v>
@@ -2066,10 +2086,10 @@
         <v>240</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H55" s="11"/>
     </row>
@@ -2078,10 +2098,10 @@
         <v>23</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D56" s="10" t="n">
         <v>50</v>
@@ -2090,10 +2110,10 @@
         <v>600</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H56" s="11"/>
     </row>
@@ -2102,10 +2122,10 @@
         <v>24</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D57" s="10" t="n">
         <v>40</v>
@@ -2114,13 +2134,13 @@
         <v>480</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2128,10 +2148,10 @@
         <v>25</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D58" s="10" t="n">
         <v>12</v>
@@ -2140,10 +2160,10 @@
         <v>144</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H58" s="11"/>
     </row>
@@ -2152,10 +2172,10 @@
         <v>26</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D59" s="10" t="n">
         <v>56</v>
@@ -2164,10 +2184,10 @@
         <v>672</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H59" s="11"/>
     </row>
@@ -2176,10 +2196,10 @@
         <v>27</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D60" s="10" t="n">
         <v>75</v>
@@ -2188,10 +2208,10 @@
         <v>900</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H60" s="11"/>
     </row>
@@ -2200,10 +2220,10 @@
         <v>28</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D61" s="10" t="n">
         <v>55</v>
@@ -2212,10 +2232,10 @@
         <v>660</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H61" s="11"/>
     </row>
@@ -2224,10 +2244,10 @@
         <v>29</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D62" s="10" t="n">
         <v>50</v>
@@ -2236,10 +2256,10 @@
         <v>600</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G62" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H62" s="11"/>
     </row>
@@ -2248,10 +2268,10 @@
         <v>30</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D63" s="10" t="n">
         <v>35</v>
@@ -2260,13 +2280,13 @@
         <v>420</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H63" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2274,10 +2294,10 @@
         <v>31</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D64" s="10" t="n">
         <v>62</v>
@@ -2286,10 +2306,10 @@
         <v>744</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G64" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H64" s="11"/>
     </row>
@@ -2298,10 +2318,10 @@
         <v>32</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D65" s="10" t="n">
         <v>42</v>
@@ -2310,10 +2330,10 @@
         <v>504</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G65" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H65" s="11"/>
     </row>
@@ -2322,10 +2342,10 @@
         <v>33</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D66" s="10" t="n">
         <v>75</v>
@@ -2334,10 +2354,10 @@
         <v>900</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G66" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H66" s="11"/>
     </row>
@@ -2346,10 +2366,10 @@
         <v>34</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D67" s="10" t="n">
         <v>75</v>
@@ -2358,10 +2378,10 @@
         <v>900</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H67" s="11"/>
     </row>
@@ -2370,10 +2390,10 @@
         <v>35</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D68" s="10" t="n">
         <v>75</v>
@@ -2382,10 +2402,10 @@
         <v>900</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H68" s="11"/>
     </row>
@@ -2394,10 +2414,10 @@
         <v>36</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D69" s="10" t="n">
         <v>40</v>
@@ -2406,10 +2426,10 @@
         <v>480</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H69" s="11"/>
     </row>
@@ -2418,10 +2438,10 @@
         <v>37</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C70" s="9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D70" s="10" t="n">
         <v>75</v>
@@ -2430,16 +2450,16 @@
         <v>900</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H70" s="11"/>
     </row>
     <row r="71" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -2449,15 +2469,15 @@
       </c>
       <c r="E71" s="7" t="n">
         <f aca="false">E13+E33</f>
-        <v>25214.008</v>
+        <v>25714.008</v>
       </c>
       <c r="F71" s="6"/>
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
     </row>
-    <row r="73" customFormat="false" ht="102.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="115.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B73" s="12"/>
       <c r="C73" s="12"/>

</xml_diff>